<commit_message>
chore: modificar plantilla arucos a 4 arucos
</commit_message>
<xml_diff>
--- a/arucos_de_prueba/PLANTILLA_ARUCOS_LARGO_ALTO_ANCHO.xlsx
+++ b/arucos_de_prueba/PLANTILLA_ARUCOS_LARGO_ALTO_ANCHO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yeferson\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C740E22-508C-4E95-9913-4BDA75CC3422}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7E574D3-8D7E-410B-B9A2-63FD83A58932}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CF2083FA-A8C9-47EF-BA1B-C6C648F5AA55}"/>
+    <workbookView xWindow="5475" yWindow="3585" windowWidth="28800" windowHeight="15345" xr2:uid="{CF2083FA-A8C9-47EF-BA1B-C6C648F5AA55}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -69,8 +69,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -93,22 +94,22 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>266964</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>22476</xdr:rowOff>
+      <xdr:colOff>266692</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>68627</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>13</xdr:col>
-      <xdr:colOff>419365</xdr:colOff>
-      <xdr:row>108</xdr:row>
-      <xdr:rowOff>95702</xdr:rowOff>
+      <xdr:colOff>419092</xdr:colOff>
+      <xdr:row>107</xdr:row>
+      <xdr:rowOff>62249</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="2" name="Grupo 1">
+        <xdr:cNvPr id="19" name="Grupo 18">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CFAA2603-610E-DC0D-60B9-E228675D3FB3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{603BCBA4-0F4D-491E-49DB-0985E9765EED}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -116,18 +117,18 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="266964" y="593976"/>
-          <a:ext cx="10058401" cy="20075726"/>
-          <a:chOff x="215010" y="1892840"/>
-          <a:chExt cx="10058401" cy="20075726"/>
+          <a:off x="266692" y="259127"/>
+          <a:ext cx="10058400" cy="20186622"/>
+          <a:chOff x="266692" y="259127"/>
+          <a:chExt cx="10058400" cy="20186622"/>
         </a:xfrm>
       </xdr:grpSpPr>
       <xdr:grpSp>
         <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="10" name="Grupo 9">
+          <xdr:cNvPr id="13" name="Grupo 12">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BAFC317F-ED02-5A37-7366-B41524FAB0AB}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B719B0C2-4865-5E83-954A-8FB951EA16EE}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
@@ -135,21 +136,18 @@
         </xdr:nvGrpSpPr>
         <xdr:grpSpPr>
           <a:xfrm>
-            <a:off x="215010" y="1892840"/>
-            <a:ext cx="10058401" cy="20075726"/>
-            <a:chOff x="1997544" y="586550"/>
-            <a:chExt cx="10058401" cy="20075726"/>
+            <a:off x="266692" y="259127"/>
+            <a:ext cx="10058400" cy="20125630"/>
+            <a:chOff x="6240442" y="588169"/>
+            <a:chExt cx="10058400" cy="20125630"/>
           </a:xfrm>
         </xdr:grpSpPr>
         <xdr:pic>
           <xdr:nvPicPr>
-            <xdr:cNvPr id="3" name="Imagen 2">
+            <xdr:cNvPr id="8" name="Imagen 7">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E54CB1AA-1FA6-35EC-95D1-397CA15F083C}"/>
-                </a:ext>
-                <a:ext uri="{C183D7F6-B498-43B3-948B-1728B52AA6E4}">
-                  <adec:decorative xmlns:adec="http://schemas.microsoft.com/office/drawing/2017/decorative" val="0"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85BE1C58-2E13-ABD0-6DEE-678E15F733FC}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -170,9 +168,9 @@
             </a:stretch>
           </xdr:blipFill>
           <xdr:spPr>
-            <a:xfrm>
-              <a:off x="1997544" y="10603876"/>
-              <a:ext cx="1057077" cy="10058400"/>
+            <a:xfrm rot="16200000">
+              <a:off x="10941001" y="5956488"/>
+              <a:ext cx="657281" cy="10058400"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -181,10 +179,10 @@
         </xdr:pic>
         <xdr:pic>
           <xdr:nvPicPr>
-            <xdr:cNvPr id="7" name="Imagen 6">
+            <xdr:cNvPr id="12" name="Imagen 11">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{67229F3B-A8B9-5DA9-F38E-9F0C22F40B62}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1E8C83EA-99FC-FDA7-84FE-4469D2D328B3}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -192,7 +190,7 @@
               <a:picLocks noChangeAspect="1"/>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
-          <xdr:blipFill rotWithShape="1">
+          <xdr:blipFill>
             <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
               <a:extLst>
                 <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
@@ -200,13 +198,14 @@
                 </a:ext>
               </a:extLst>
             </a:blip>
-            <a:srcRect l="1876" r="2266"/>
-            <a:stretch/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
           </xdr:blipFill>
           <xdr:spPr>
-            <a:xfrm rot="16200000">
-              <a:off x="6520097" y="6103756"/>
-              <a:ext cx="1013296" cy="10058400"/>
+            <a:xfrm rot="10800000">
+              <a:off x="6244828" y="588169"/>
+              <a:ext cx="657281" cy="10058400"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -215,10 +214,10 @@
         </xdr:pic>
         <xdr:pic>
           <xdr:nvPicPr>
-            <xdr:cNvPr id="9" name="Imagen 8">
+            <xdr:cNvPr id="5" name="Imagen 4">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B2229FF-8B9F-BC19-3FDD-B5551C801F62}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E224A255-CBE5-328F-DBEA-7AED5E1DE1D2}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -226,22 +225,22 @@
               <a:picLocks noChangeAspect="1"/>
             </xdr:cNvPicPr>
           </xdr:nvPicPr>
-          <xdr:blipFill rotWithShape="1">
+          <xdr:blipFill>
             <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-              <a:alphaModFix/>
               <a:extLst>
                 <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
                   <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
                 </a:ext>
               </a:extLst>
             </a:blip>
-            <a:srcRect l="2122" t="203" r="383" b="25"/>
-            <a:stretch/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
           </xdr:blipFill>
           <xdr:spPr>
-            <a:xfrm rot="10800000">
-              <a:off x="2021670" y="586550"/>
-              <a:ext cx="1030597" cy="10035702"/>
+            <a:xfrm>
+              <a:off x="6241816" y="10655399"/>
+              <a:ext cx="657281" cy="10058400"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -251,19 +250,19 @@
       </xdr:grpSp>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="32" name="CuadroTexto 31">
+          <xdr:cNvPr id="14" name="CuadroTexto 13">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CFD36570-7D2E-2052-308E-ACF6B2C99F25}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F71B31BB-027F-9B53-8240-65E52A5B596E}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
           <xdr:cNvSpPr txBox="1"/>
         </xdr:nvSpPr>
         <xdr:spPr>
-          <a:xfrm>
-            <a:off x="1351871" y="12961654"/>
-            <a:ext cx="8677953" cy="170624"/>
+          <a:xfrm rot="5400000">
+            <a:off x="-3333468" y="15859718"/>
+            <a:ext cx="9001439" cy="170624"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -290,33 +289,156 @@
           </a:bodyPr>
           <a:lstStyle/>
           <a:p>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
             <a:r>
               <a:rPr lang="es-CL" sz="500"/>
-              <a:t>LARGO1</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="es-CL" sz="500" baseline="0"/>
-              <a:t>	LARGO2	LARGO3	LARGO4	LARGO5	LARGO6	LARGO7	LARGO8	LARGO9	LARGO10</a:t>
-            </a:r>
-            <a:endParaRPr lang="es-CL" sz="500"/>
+              <a:t>ANCHO 1 ID 0-199	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ANCHO 2 ID 0-199</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t> 	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ANCHO 3 ID 0-199</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ANCHO 4 ID 0-199	ANCHO 5 ID 0-199	ANCHO 6 ID 0-199	ANCHO 7 ID 0-199</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t> 	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ANCHO 8 ID 0-199</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ANCHO 9 ID 0-199	ANCHO 10 ID 0-199</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-CL" sz="500">
+              <a:effectLst/>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="33" name="CuadroTexto 32">
+          <xdr:cNvPr id="17" name="CuadroTexto 16">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B801D13C-C209-4A40-B958-D23EDBC1A754}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{179C8834-8B92-4369-BB18-DE1E4ED65E5B}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
           <xdr:cNvSpPr txBox="1"/>
         </xdr:nvSpPr>
         <xdr:spPr>
-          <a:xfrm rot="16200000">
-            <a:off x="-2990336" y="17384775"/>
-            <a:ext cx="8695009" cy="170624"/>
+          <a:xfrm>
+            <a:off x="1048171" y="11118407"/>
+            <a:ext cx="9049400" cy="170624"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -343,9 +465,38 @@
           </a:bodyPr>
           <a:lstStyle/>
           <a:p>
-            <a:r>
-              <a:rPr lang="es-CL" sz="500" baseline="0"/>
-              <a:t>ANCHO10	ANCHO9	ANCHO8	ANCHO7	ANCHO6	</a:t>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500"/>
+              <a:t>LARGO 1 ID 200-399	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>LARGO 2 ID 200-399</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="es-CL" sz="500" baseline="0">
@@ -357,27 +508,113 @@
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:rPr>
-              <a:t>ANCHO5	ANCHO4	ANCHO3	ANCHO2	ANCHO1</a:t>
-            </a:r>
-            <a:endParaRPr lang="es-CL" sz="500"/>
+              <a:t> 	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>LARGO 3 ID 200-399</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>LARGO 4 ID 200-399	LARGO 5 ID 200-399	LARGO 6 ID 200-399	LARGO 7 ID 200-399</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t> 	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>LARGO 8 ID 200-399</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>LARGO 9 ID 200-399	LARGO 10 ID 200-399</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-CL" sz="500">
+              <a:effectLst/>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
       <xdr:sp macro="" textlink="">
         <xdr:nvSpPr>
-          <xdr:cNvPr id="34" name="CuadroTexto 33">
+          <xdr:cNvPr id="18" name="CuadroTexto 17">
             <a:extLst>
               <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55A03EAA-FDA6-4BE0-ABE7-F54015BE0CC3}"/>
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AF3815B0-02A2-4210-AA73-A2FA77850215}"/>
               </a:ext>
             </a:extLst>
           </xdr:cNvPr>
           <xdr:cNvSpPr txBox="1"/>
         </xdr:nvSpPr>
         <xdr:spPr>
-          <a:xfrm rot="16200000">
-            <a:off x="-3415632" y="6952001"/>
-            <a:ext cx="9552230" cy="170624"/>
+          <a:xfrm rot="5400000">
+            <a:off x="-3332923" y="5299822"/>
+            <a:ext cx="9000349" cy="170624"/>
           </a:xfrm>
           <a:prstGeom prst="rect">
             <a:avLst/>
@@ -404,9 +641,38 @@
           </a:bodyPr>
           <a:lstStyle/>
           <a:p>
-            <a:r>
-              <a:rPr lang="es-CL" sz="500" baseline="0"/>
-              <a:t>ALTO1	ALTO2	ALTO3	ALTO4	ALTO5	</a:t>
+            <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+              <a:lnSpc>
+                <a:spcPct val="100000"/>
+              </a:lnSpc>
+              <a:spcBef>
+                <a:spcPts val="0"/>
+              </a:spcBef>
+              <a:spcAft>
+                <a:spcPts val="0"/>
+              </a:spcAft>
+              <a:buClrTx/>
+              <a:buSzTx/>
+              <a:buFontTx/>
+              <a:buNone/>
+              <a:tabLst/>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500"/>
+              <a:t>ALTO 1 ID 400-599	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ALTO 2 ID 400-599</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="es-CL" sz="500" baseline="0">
@@ -418,177 +684,95 @@
                 <a:ea typeface="+mn-ea"/>
                 <a:cs typeface="+mn-cs"/>
               </a:rPr>
-              <a:t>ALTO6	ALTO7	ALTO8	ALTO9	ALTO10	ALTO11</a:t>
-            </a:r>
-            <a:endParaRPr lang="es-CL" sz="500"/>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="35" name="CuadroTexto 34">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{98DC3499-EB45-DEE9-1BC1-ABD9FCCF42ED}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr txBox="1"/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm rot="16200000">
-            <a:off x="1092196" y="13725812"/>
-            <a:ext cx="704001" cy="342786"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:lnRef>
-          <a:fillRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="tx1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr">
-            <a:spAutoFit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="es-CL" sz="800"/>
-              <a:t>IDS</a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="es-CL" sz="800"/>
-              <a:t>0-299</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="36" name="CuadroTexto 35">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{252ECECE-554D-4667-9C08-D7199FF05453}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr txBox="1"/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="1645304" y="11585643"/>
-            <a:ext cx="704001" cy="342786"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:lnRef>
-          <a:fillRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="tx1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr">
-            <a:spAutoFit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="es-CL" sz="800"/>
-              <a:t>IDS</a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="es-CL" sz="800"/>
-              <a:t>300-599</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="37" name="CuadroTexto 36">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{342E296D-C291-4762-9265-1D7878DBDBED}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr txBox="1"/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm rot="16200000">
-            <a:off x="1070559" y="10984544"/>
-            <a:ext cx="704001" cy="342786"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:lnRef>
-          <a:fillRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:scrgbClr r="0" g="0" b="0"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="tx1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr">
-            <a:spAutoFit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="es-CL" sz="800"/>
-              <a:t>IDS</a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="es-CL" sz="800"/>
-              <a:t>600-899</a:t>
-            </a:r>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ALTO 3 ID 400-599</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ALTO 4 ID 400-599	ALTO 5 ID 400-599	ALTO 6 ID 400-599	ALTO 7 ID 400-599</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ALTO 8 ID 400-599</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>	</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CL" sz="500">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:effectLst/>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:rPr>
+              <a:t>ALTO 9 ID 400-599	ALTO 10 ID 400-599</a:t>
+            </a:r>
+            <a:endParaRPr lang="es-CL" sz="500">
+              <a:effectLst/>
+            </a:endParaRPr>
           </a:p>
         </xdr:txBody>
       </xdr:sp>
@@ -917,6 +1101,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D7B5996-CFD9-4D78-9871-C2CB1B8965D3}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="16384" width="11.42578125" style="1"/>
+  </cols>
   <sheetData/>
   <pageMargins left="1.1811023622047245" right="1.1811023622047245" top="1.1811023622047245" bottom="1.1811023622047245" header="1.1811023622047245" footer="0.31496062992125984"/>
   <pageSetup fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>

</xml_diff>